<commit_message>
Add session 9 notebook covering modules, imports, and error handling in Python
</commit_message>
<xml_diff>
--- a/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/01-ML4NLU-Matrix-Multiplication.xlsx
+++ b/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/01-ML4NLU-Matrix-Multiplication.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/peye9704_colorado_edu/Documents/2024/AIbyHand/spreadsheets/github/ai-by-hand-excel/workbook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hd/Desktop/Machine Learning/ML-Excercises/Excels/Lecture_Machine_Learning_for_Natural_Language_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{5D0C14FE-EDCB-D849-B8A8-6E2FA0AF1751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1852AA40-8C8A-2D42-8AF1-FC4C998AC48B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1A1D7D0-AE12-004C-9371-59710DCA3A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17540" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17540" activeTab="3" xr2:uid="{045A32B7-7D49-AA41-9BCB-690BF8CB81ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Exrcise 1-5" sheetId="1" r:id="rId1"/>
@@ -1050,30 +1050,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1086,6 +1062,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1107,12 +1089,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1129,6 +1129,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1150,15 +1159,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1525,7 +1525,7 @@
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="str">
         <f>IF(ISBLANK(F9)=TRUE,"NOT DONE",IF(B5=F9,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -1534,7 +1534,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
         <f>IF(ISBLANK(L10)=TRUE,"NOT DONE",IF(H5=L10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -1543,21 +1543,21 @@
     </row>
     <row r="4" spans="1:15" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
-      <c r="B4" s="111" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="112"/>
-      <c r="D4" s="112"/>
-      <c r="E4" s="112"/>
-      <c r="F4" s="113"/>
+      <c r="B4" s="103" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="105"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="111" t="s">
+      <c r="H4" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="112"/>
-      <c r="J4" s="112"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="113"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="105"/>
     </row>
     <row r="5" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
@@ -1582,16 +1582,16 @@
       <c r="B6" s="4"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="108" t="s">
+      <c r="E6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="109"/>
+      <c r="F6" s="107"/>
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
-      <c r="K6" s="108" t="s">
+      <c r="K6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="L6" s="109"/>
+      <c r="L6" s="107"/>
     </row>
     <row r="7" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
@@ -1648,9 +1648,11 @@
         <f>C9*E7</f>
         <v>15</v>
       </c>
-      <c r="F9" s="20"/>
+      <c r="F9" s="20">
+        <v>6</v>
+      </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="110" t="s">
+      <c r="H9" s="102" t="s">
         <v>47</v>
       </c>
       <c r="I9" s="19">
@@ -1671,12 +1673,12 @@
       <c r="B10" s="8"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="103"/>
+      <c r="F10" s="116"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="110"/>
+      <c r="H10" s="102"/>
       <c r="I10" s="19">
         <v>2</v>
       </c>
@@ -1687,7 +1689,9 @@
         <f>I10*K7</f>
         <v>4</v>
       </c>
-      <c r="L10" s="21"/>
+      <c r="L10" s="21">
+        <v>-4</v>
+      </c>
     </row>
     <row r="11" spans="1:15" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
@@ -1700,10 +1704,10 @@
       <c r="H11" s="8"/>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
-      <c r="K11" s="102" t="s">
+      <c r="K11" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="L11" s="103"/>
+      <c r="L11" s="116"/>
     </row>
     <row r="12" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -1737,7 +1741,7 @@
       <c r="A14" s="3"/>
       <c r="B14" s="3" t="str">
         <f>IF(ISBLANK(F21)=TRUE,"NOT DONE",IF(B16=F21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1746,7 +1750,7 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="str">
         <f>IF(ISBLANK(I21)=TRUE,"NOT DONE",IF(H16=I21,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="I14" s="27"/>
       <c r="J14" s="27"/>
@@ -1755,21 +1759,21 @@
     </row>
     <row r="15" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
-      <c r="B15" s="111" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="112"/>
-      <c r="D15" s="112"/>
-      <c r="E15" s="112"/>
-      <c r="F15" s="113"/>
+      <c r="B15" s="103" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="104"/>
+      <c r="D15" s="104"/>
+      <c r="E15" s="104"/>
+      <c r="F15" s="105"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="114" t="s">
+      <c r="H15" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="115"/>
-      <c r="J15" s="115"/>
-      <c r="K15" s="115"/>
-      <c r="L15" s="116"/>
+      <c r="I15" s="109"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="109"/>
+      <c r="L15" s="110"/>
     </row>
     <row r="16" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
@@ -1804,10 +1808,10 @@
       <c r="H17" s="4"/>
       <c r="I17" s="29"/>
       <c r="J17" s="29"/>
-      <c r="K17" s="117" t="s">
+      <c r="K17" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="L17" s="118"/>
+      <c r="L17" s="112"/>
     </row>
     <row r="18" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
@@ -1851,7 +1855,7 @@
     </row>
     <row r="20" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
-      <c r="B20" s="120" t="s">
+      <c r="B20" s="114" t="s">
         <v>47</v>
       </c>
       <c r="C20" s="19">
@@ -1864,7 +1868,7 @@
         <v>12</v>
       </c>
       <c r="G20" s="3"/>
-      <c r="H20" s="119" t="s">
+      <c r="H20" s="113" t="s">
         <v>47</v>
       </c>
       <c r="I20" s="35">
@@ -1882,18 +1886,22 @@
     </row>
     <row r="21" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
-      <c r="B21" s="120"/>
+      <c r="B21" s="114"/>
       <c r="C21" s="19">
         <v>2</v>
       </c>
-      <c r="D21" s="104" t="s">
+      <c r="D21" s="117" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="105"/>
-      <c r="F21" s="21"/>
+      <c r="E21" s="118"/>
+      <c r="F21" s="21">
+        <v>8</v>
+      </c>
       <c r="G21" s="3"/>
-      <c r="H21" s="119"/>
-      <c r="I21" s="42"/>
+      <c r="H21" s="113"/>
+      <c r="I21" s="42">
+        <v>0</v>
+      </c>
       <c r="J21" s="38" t="s">
         <v>44</v>
       </c>
@@ -1917,10 +1925,10 @@
       <c r="H22" s="40"/>
       <c r="I22" s="41"/>
       <c r="J22" s="41"/>
-      <c r="K22" s="106" t="s">
+      <c r="K22" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="L22" s="107"/>
+      <c r="L22" s="120"/>
     </row>
     <row r="23" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
@@ -1954,7 +1962,7 @@
       <c r="A25" s="3"/>
       <c r="B25" s="3" t="str">
         <f>IF(ISBLANK(F32)=TRUE,"NOT DONE",IF(B27=F32,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1969,13 +1977,13 @@
     </row>
     <row r="26" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
-      <c r="B26" s="111" t="s">
+      <c r="B26" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="C26" s="112"/>
-      <c r="D26" s="112"/>
-      <c r="E26" s="112"/>
-      <c r="F26" s="113"/>
+      <c r="C26" s="104"/>
+      <c r="D26" s="104"/>
+      <c r="E26" s="104"/>
+      <c r="F26" s="105"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
@@ -2001,10 +2009,10 @@
     <row r="28" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
-      <c r="E28" s="108" t="s">
+      <c r="E28" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="F28" s="109"/>
+      <c r="F28" s="107"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -2048,7 +2056,7 @@
     </row>
     <row r="31" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
-      <c r="B31" s="110" t="s">
+      <c r="B31" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C31" s="19">
@@ -2072,7 +2080,7 @@
     </row>
     <row r="32" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
-      <c r="B32" s="110"/>
+      <c r="B32" s="102"/>
       <c r="C32" s="19">
         <v>-1</v>
       </c>
@@ -2083,7 +2091,9 @@
         <f>C32*E29</f>
         <v>-1</v>
       </c>
-      <c r="F32" s="21"/>
+      <c r="F32" s="21">
+        <v>1</v>
+      </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
@@ -2096,10 +2106,10 @@
       <c r="B33" s="8"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
-      <c r="E33" s="102" t="s">
+      <c r="E33" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="F33" s="103"/>
+      <c r="F33" s="116"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
@@ -2109,6 +2119,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="B31:B32"/>
     <mergeCell ref="H4:L4"/>
     <mergeCell ref="K6:L6"/>
@@ -2121,12 +2137,6 @@
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="B20:B21"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="E28:F28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O1" r:id="rId1" xr:uid="{5D80921D-A4FC-D544-B52C-2180A5E1740E}"/>
@@ -2172,7 +2182,7 @@
     <row r="3" spans="1:17" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C3" s="3" t="str">
         <f>IF(ISBLANK(D10)=TRUE,"NOT DONE",IF(B5=D10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="D3" s="27"/>
       <c r="E3" s="27"/>
@@ -2180,7 +2190,7 @@
       <c r="G3" s="27"/>
       <c r="I3" s="3" t="str">
         <f>IF(ISBLANK(M11)=TRUE,"NOT DONE",IF(I5=M11,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="27"/>
@@ -2189,22 +2199,22 @@
       <c r="N3" s="27"/>
     </row>
     <row r="4" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="C4" s="114" t="s">
+      <c r="C4" s="108" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="122"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="109"/>
+      <c r="F4" s="109"/>
+      <c r="G4" s="121"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="114" t="s">
+      <c r="I4" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="122"/>
+      <c r="J4" s="109"/>
+      <c r="K4" s="109"/>
+      <c r="L4" s="109"/>
+      <c r="M4" s="109"/>
+      <c r="N4" s="121"/>
     </row>
     <row r="5" spans="1:17" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="45">
@@ -2232,19 +2242,19 @@
       <c r="C6" s="4"/>
       <c r="D6" s="29"/>
       <c r="E6" s="29"/>
-      <c r="F6" s="117" t="s">
+      <c r="F6" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="121"/>
+      <c r="G6" s="122"/>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
       <c r="J6" s="3"/>
       <c r="K6" s="29"/>
       <c r="L6" s="29"/>
-      <c r="M6" s="117" t="s">
+      <c r="M6" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="N6" s="121"/>
+      <c r="N6" s="122"/>
     </row>
     <row r="7" spans="1:17" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="27"/>
@@ -2293,7 +2303,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="C9" s="119" t="s">
+      <c r="C9" s="113" t="s">
         <v>47</v>
       </c>
       <c r="D9" s="35">
@@ -2319,8 +2329,10 @@
       <c r="N9" s="34"/>
     </row>
     <row r="10" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="C10" s="119"/>
-      <c r="D10" s="42"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="42">
+        <v>-1</v>
+      </c>
       <c r="E10" s="38" t="s">
         <v>44</v>
       </c>
@@ -2331,7 +2343,7 @@
         <v>2</v>
       </c>
       <c r="H10" s="3"/>
-      <c r="I10" s="119" t="s">
+      <c r="I10" s="113" t="s">
         <v>47</v>
       </c>
       <c r="J10" s="47">
@@ -2355,12 +2367,12 @@
       <c r="C11" s="40"/>
       <c r="D11" s="41"/>
       <c r="E11" s="41"/>
-      <c r="F11" s="106" t="s">
+      <c r="F11" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="107"/>
+      <c r="G11" s="120"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="119"/>
+      <c r="I11" s="113"/>
       <c r="J11" s="47">
         <v>4</v>
       </c>
@@ -2370,7 +2382,9 @@
       <c r="L11" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="M11" s="49"/>
+      <c r="M11" s="49">
+        <v>-1</v>
+      </c>
       <c r="N11" s="43">
         <f>J11*N7+K11*N8</f>
         <v>9</v>
@@ -2388,10 +2402,10 @@
       <c r="J12" s="41"/>
       <c r="K12" s="41"/>
       <c r="L12" s="41"/>
-      <c r="M12" s="106" t="s">
+      <c r="M12" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="N12" s="107"/>
+      <c r="N12" s="120"/>
     </row>
     <row r="13" spans="1:17" ht="19" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
@@ -2425,7 +2439,7 @@
     <row r="15" spans="1:17" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="str">
         <f>IF(ISBLANK(G22)=TRUE,"NOT DONE",IF(B17=G22,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="27"/>
@@ -2435,7 +2449,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="3" t="str">
         <f>IF(ISBLANK(M23)=TRUE,"NOT DONE",IF(I17=M23,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="27"/>
@@ -2444,23 +2458,23 @@
       <c r="N15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="B16" s="114" t="s">
+      <c r="B16" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="115"/>
-      <c r="D16" s="115"/>
-      <c r="E16" s="115"/>
-      <c r="F16" s="115"/>
-      <c r="G16" s="122"/>
+      <c r="C16" s="109"/>
+      <c r="D16" s="109"/>
+      <c r="E16" s="109"/>
+      <c r="F16" s="109"/>
+      <c r="G16" s="121"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="114" t="s">
+      <c r="I16" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="J16" s="115"/>
-      <c r="K16" s="115"/>
-      <c r="L16" s="115"/>
-      <c r="M16" s="115"/>
-      <c r="N16" s="122"/>
+      <c r="J16" s="109"/>
+      <c r="K16" s="109"/>
+      <c r="L16" s="109"/>
+      <c r="M16" s="109"/>
+      <c r="N16" s="121"/>
     </row>
     <row r="17" spans="2:14" ht="19" x14ac:dyDescent="0.25">
       <c r="B17" s="18">
@@ -2488,19 +2502,19 @@
       <c r="C18" s="3"/>
       <c r="D18" s="29"/>
       <c r="E18" s="29"/>
-      <c r="F18" s="117" t="s">
+      <c r="F18" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="G18" s="121"/>
+      <c r="G18" s="122"/>
       <c r="H18" s="3"/>
       <c r="I18" s="4"/>
       <c r="J18" s="3"/>
       <c r="K18" s="29"/>
       <c r="L18" s="29"/>
-      <c r="M18" s="117" t="s">
+      <c r="M18" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="N18" s="121"/>
+      <c r="N18" s="122"/>
     </row>
     <row r="19" spans="2:14" ht="19" x14ac:dyDescent="0.25">
       <c r="B19" s="31"/>
@@ -2568,7 +2582,7 @@
       <c r="N21" s="34"/>
     </row>
     <row r="22" spans="2:14" ht="19" x14ac:dyDescent="0.25">
-      <c r="B22" s="119" t="s">
+      <c r="B22" s="113" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="47">
@@ -2584,9 +2598,11 @@
         <f>C22*F19+D22*F20</f>
         <v>4</v>
       </c>
-      <c r="G22" s="65"/>
+      <c r="G22" s="65">
+        <v>5</v>
+      </c>
       <c r="H22" s="3"/>
-      <c r="I22" s="119" t="s">
+      <c r="I22" s="113" t="s">
         <v>47</v>
       </c>
       <c r="J22" s="47">
@@ -2606,7 +2622,7 @@
       </c>
     </row>
     <row r="23" spans="2:14" ht="19" x14ac:dyDescent="0.25">
-      <c r="B23" s="119"/>
+      <c r="B23" s="113"/>
       <c r="C23" s="47">
         <v>1</v>
       </c>
@@ -2623,7 +2639,7 @@
         <v>1</v>
       </c>
       <c r="H23" s="3"/>
-      <c r="I23" s="119"/>
+      <c r="I23" s="113"/>
       <c r="J23" s="47">
         <v>-2</v>
       </c>
@@ -2633,7 +2649,9 @@
       <c r="L23" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="M23" s="49"/>
+      <c r="M23" s="49">
+        <v>-4</v>
+      </c>
       <c r="N23" s="43">
         <f>J23*N19+K23*N20</f>
         <v>0</v>
@@ -2644,19 +2662,19 @@
       <c r="C24" s="41"/>
       <c r="D24" s="41"/>
       <c r="E24" s="41"/>
-      <c r="F24" s="106" t="s">
+      <c r="F24" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="G24" s="107"/>
+      <c r="G24" s="120"/>
       <c r="H24" s="3"/>
       <c r="I24" s="40"/>
       <c r="J24" s="41"/>
       <c r="K24" s="41"/>
       <c r="L24" s="41"/>
-      <c r="M24" s="106" t="s">
+      <c r="M24" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="N24" s="107"/>
+      <c r="N24" s="120"/>
     </row>
     <row r="25" spans="2:14" ht="19" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
@@ -2689,7 +2707,7 @@
     <row r="27" spans="2:14" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="str">
         <f>IF(ISBLANK(F35)=TRUE,"NOT DONE",IF(B29=F35,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="27"/>
@@ -2704,14 +2722,14 @@
       <c r="M27" s="3"/>
     </row>
     <row r="28" spans="2:14" ht="19" x14ac:dyDescent="0.25">
-      <c r="B28" s="114" t="s">
+      <c r="B28" s="108" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="115"/>
-      <c r="D28" s="115"/>
-      <c r="E28" s="115"/>
-      <c r="F28" s="115"/>
-      <c r="G28" s="122"/>
+      <c r="C28" s="109"/>
+      <c r="D28" s="109"/>
+      <c r="E28" s="109"/>
+      <c r="F28" s="109"/>
+      <c r="G28" s="121"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
@@ -2741,10 +2759,10 @@
       <c r="C30" s="3"/>
       <c r="D30" s="29"/>
       <c r="E30" s="29"/>
-      <c r="F30" s="117" t="s">
+      <c r="F30" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="G30" s="121"/>
+      <c r="G30" s="122"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -2805,7 +2823,7 @@
       <c r="M33" s="3"/>
     </row>
     <row r="34" spans="2:13" ht="19" x14ac:dyDescent="0.25">
-      <c r="B34" s="119" t="s">
+      <c r="B34" s="113" t="s">
         <v>47</v>
       </c>
       <c r="C34" s="47">
@@ -2825,7 +2843,7 @@
       </c>
     </row>
     <row r="35" spans="2:13" ht="19" x14ac:dyDescent="0.25">
-      <c r="B35" s="119"/>
+      <c r="B35" s="113"/>
       <c r="C35" s="47">
         <v>1</v>
       </c>
@@ -2835,7 +2853,9 @@
       <c r="E35" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="F35" s="49"/>
+      <c r="F35" s="49">
+        <v>-2</v>
+      </c>
       <c r="G35" s="43">
         <f>C35*G31+D35*G32</f>
         <v>2</v>
@@ -2846,13 +2866,24 @@
       <c r="C36" s="41"/>
       <c r="D36" s="41"/>
       <c r="E36" s="41"/>
-      <c r="F36" s="106" t="s">
+      <c r="F36" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="G36" s="107"/>
+      <c r="G36" s="120"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="I16:N16"/>
+    <mergeCell ref="M18:N18"/>
     <mergeCell ref="C4:G4"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="F24:G24"/>
@@ -2862,17 +2893,6 @@
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="F18:G18"/>
     <mergeCell ref="B22:B23"/>
-    <mergeCell ref="I4:N4"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="I16:N16"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="I22:I23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q1" r:id="rId1" xr:uid="{5546FD2C-4841-294A-8FD0-6BC005E41B70}"/>
@@ -2922,7 +2942,7 @@
     <row r="3" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="str">
         <f>IF(ISBLANK(H10)=TRUE,"NOT DONE",IF(B5=H10,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="27"/>
@@ -2933,21 +2953,21 @@
       <c r="I3" s="27"/>
       <c r="K3" t="str">
         <f>IF(ISBLANK(P11)=TRUE,"NOT DONE",IF(K5=P11,"CORRECT","INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="19" x14ac:dyDescent="0.25">
-      <c r="B4" s="114" t="s">
+      <c r="B4" s="108" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="115"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="122"/>
-      <c r="K4" s="111" t="s">
+      <c r="C4" s="109"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="109"/>
+      <c r="F4" s="109"/>
+      <c r="G4" s="109"/>
+      <c r="H4" s="109"/>
+      <c r="I4" s="121"/>
+      <c r="K4" s="103" t="s">
         <v>13</v>
       </c>
       <c r="L4" s="123"/>
@@ -2984,20 +3004,20 @@
       <c r="C6" s="3"/>
       <c r="D6" s="29"/>
       <c r="E6" s="29"/>
-      <c r="F6" s="117" t="s">
+      <c r="F6" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="117"/>
-      <c r="H6" s="117"/>
-      <c r="I6" s="121"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="122"/>
       <c r="K6" s="4"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="P6" s="108" t="s">
+      <c r="P6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="Q6" s="109"/>
+      <c r="Q6" s="107"/>
     </row>
     <row r="7" spans="1:19" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="31"/>
@@ -3078,7 +3098,7 @@
       </c>
     </row>
     <row r="10" spans="1:19" ht="19" x14ac:dyDescent="0.25">
-      <c r="B10" s="119" t="s">
+      <c r="B10" s="113" t="s">
         <v>47</v>
       </c>
       <c r="C10" s="47">
@@ -3098,7 +3118,9 @@
         <f>C10*G7+D10*G8</f>
         <v>4</v>
       </c>
-      <c r="H10" s="46"/>
+      <c r="H10" s="46">
+        <v>-2</v>
+      </c>
       <c r="I10" s="50">
         <f>C10*I7+D10*I8</f>
         <v>-4</v>
@@ -3113,7 +3135,7 @@
       <c r="Q10" s="71"/>
     </row>
     <row r="11" spans="1:19" ht="19" x14ac:dyDescent="0.25">
-      <c r="B11" s="119"/>
+      <c r="B11" s="113"/>
       <c r="C11" s="47">
         <v>2</v>
       </c>
@@ -3137,7 +3159,7 @@
         <f>I7*C11+I8*D11</f>
         <v>-6</v>
       </c>
-      <c r="K11" s="110" t="s">
+      <c r="K11" s="102" t="s">
         <v>47</v>
       </c>
       <c r="L11" s="19">
@@ -3152,7 +3174,9 @@
       <c r="O11" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="P11" s="69"/>
+      <c r="P11" s="69">
+        <v>6</v>
+      </c>
       <c r="Q11" s="75">
         <f>L11*Q7+M11*Q8+N11*Q9</f>
         <v>2</v>
@@ -3163,13 +3187,13 @@
       <c r="C12" s="41"/>
       <c r="D12" s="41"/>
       <c r="E12" s="41"/>
-      <c r="F12" s="106" t="s">
+      <c r="F12" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="G12" s="106"/>
-      <c r="H12" s="106"/>
-      <c r="I12" s="107"/>
-      <c r="K12" s="110"/>
+      <c r="G12" s="119"/>
+      <c r="H12" s="119"/>
+      <c r="I12" s="120"/>
+      <c r="K12" s="102"/>
       <c r="L12" s="59">
         <v>2</v>
       </c>
@@ -3203,10 +3227,10 @@
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
       <c r="O13" s="72"/>
-      <c r="P13" s="102" t="s">
+      <c r="P13" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="Q13" s="103"/>
+      <c r="Q13" s="116"/>
     </row>
     <row r="14" spans="1:19" ht="19" x14ac:dyDescent="0.25">
       <c r="B14" s="27"/>
@@ -3227,7 +3251,7 @@
     <row r="16" spans="1:19" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="str">
         <f>IF(ISBLANK(H24)=TRUE,"NOT DONE",IF(B18=H24,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="27"/>
@@ -3238,7 +3262,7 @@
       <c r="I16" s="27"/>
       <c r="K16" s="3" t="str">
         <f>IF(ISBLANK(P25)=TRUE,"NOT DONE",IF(K18=P25,"CORRECT", "INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
       <c r="L16" s="3"/>
       <c r="M16" s="27"/>
@@ -3249,25 +3273,25 @@
       <c r="R16" s="27"/>
     </row>
     <row r="17" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B17" s="114" t="s">
+      <c r="B17" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="115"/>
-      <c r="D17" s="115"/>
-      <c r="E17" s="115"/>
-      <c r="F17" s="115"/>
-      <c r="G17" s="115"/>
-      <c r="H17" s="115"/>
-      <c r="I17" s="122"/>
-      <c r="K17" s="114" t="s">
+      <c r="C17" s="109"/>
+      <c r="D17" s="109"/>
+      <c r="E17" s="109"/>
+      <c r="F17" s="109"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="121"/>
+      <c r="K17" s="108" t="s">
         <v>14</v>
       </c>
-      <c r="L17" s="115"/>
-      <c r="M17" s="115"/>
-      <c r="N17" s="115"/>
-      <c r="O17" s="115"/>
-      <c r="P17" s="115"/>
-      <c r="Q17" s="122"/>
+      <c r="L17" s="109"/>
+      <c r="M17" s="109"/>
+      <c r="N17" s="109"/>
+      <c r="O17" s="109"/>
+      <c r="P17" s="109"/>
+      <c r="Q17" s="121"/>
       <c r="R17" s="29"/>
     </row>
     <row r="18" spans="2:18" ht="19" x14ac:dyDescent="0.25">
@@ -3299,21 +3323,21 @@
       <c r="C19" s="3"/>
       <c r="D19" s="29"/>
       <c r="E19" s="29"/>
-      <c r="F19" s="117" t="s">
+      <c r="F19" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="G19" s="117"/>
-      <c r="H19" s="117"/>
-      <c r="I19" s="121"/>
+      <c r="G19" s="111"/>
+      <c r="H19" s="111"/>
+      <c r="I19" s="122"/>
       <c r="K19" s="4"/>
       <c r="L19" s="3"/>
       <c r="M19" s="29"/>
       <c r="N19" s="29"/>
-      <c r="O19" s="117" t="s">
+      <c r="O19" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="P19" s="117"/>
-      <c r="Q19" s="121"/>
+      <c r="P19" s="111"/>
+      <c r="Q19" s="122"/>
       <c r="R19" s="29"/>
     </row>
     <row r="20" spans="2:18" ht="19" x14ac:dyDescent="0.25">
@@ -3403,7 +3427,7 @@
       <c r="R22" s="29"/>
     </row>
     <row r="23" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B23" s="119" t="s">
+      <c r="B23" s="113" t="s">
         <v>47</v>
       </c>
       <c r="C23" s="36">
@@ -3429,7 +3453,7 @@
         <f>C23*I20+D23*I21</f>
         <v>3</v>
       </c>
-      <c r="K23" s="119" t="s">
+      <c r="K23" s="113" t="s">
         <v>47</v>
       </c>
       <c r="L23" s="36">
@@ -3454,7 +3478,7 @@
       <c r="R23" s="29"/>
     </row>
     <row r="24" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B24" s="119"/>
+      <c r="B24" s="113"/>
       <c r="C24" s="47">
         <v>1</v>
       </c>
@@ -3472,12 +3496,14 @@
         <f>C24*G20+D24*G21</f>
         <v>1</v>
       </c>
-      <c r="H24" s="46"/>
+      <c r="H24" s="46">
+        <v>1</v>
+      </c>
       <c r="I24" s="50">
         <f>C24*I20+D24*I21</f>
         <v>-1</v>
       </c>
-      <c r="K24" s="119"/>
+      <c r="K24" s="113"/>
       <c r="L24" s="47">
         <v>1</v>
       </c>
@@ -3500,7 +3526,7 @@
       <c r="R24" s="29"/>
     </row>
     <row r="25" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B25" s="119"/>
+      <c r="B25" s="113"/>
       <c r="C25" s="47">
         <v>1</v>
       </c>
@@ -3524,7 +3550,7 @@
         <f>I20*C25+I21*D25</f>
         <v>1</v>
       </c>
-      <c r="K25" s="119"/>
+      <c r="K25" s="113"/>
       <c r="L25" s="47">
         <v>0</v>
       </c>
@@ -3538,7 +3564,9 @@
         <f>O20*L25+O21*M25</f>
         <v>2</v>
       </c>
-      <c r="P25" s="46"/>
+      <c r="P25" s="46">
+        <v>1</v>
+      </c>
       <c r="Q25" s="78">
         <f>Q20*L25+Q21*M25</f>
         <v>3</v>
@@ -3550,21 +3578,21 @@
       <c r="C26" s="41"/>
       <c r="D26" s="41"/>
       <c r="E26" s="41"/>
-      <c r="F26" s="106" t="s">
+      <c r="F26" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="G26" s="106"/>
-      <c r="H26" s="106"/>
-      <c r="I26" s="107"/>
+      <c r="G26" s="119"/>
+      <c r="H26" s="119"/>
+      <c r="I26" s="120"/>
       <c r="K26" s="40"/>
       <c r="L26" s="41"/>
       <c r="M26" s="41"/>
       <c r="N26" s="41"/>
-      <c r="O26" s="106" t="s">
+      <c r="O26" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="P26" s="106"/>
-      <c r="Q26" s="107"/>
+      <c r="P26" s="119"/>
+      <c r="Q26" s="120"/>
       <c r="R26" s="29"/>
     </row>
     <row r="27" spans="2:18" ht="19" x14ac:dyDescent="0.25">
@@ -3581,11 +3609,11 @@
     <row r="29" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <f>IF(ISBLANK(H38)=TRUE,"NOT DONE",IF(B31=H38,"CORRECT","INCORRECT"))</f>
-        <v>NOT DONE</v>
+        <v>CORRECT</v>
       </c>
     </row>
     <row r="30" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B30" s="111" t="s">
+      <c r="B30" s="103" t="s">
         <v>12</v>
       </c>
       <c r="C30" s="123"/>
@@ -3613,10 +3641,10 @@
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="G32" s="108" t="s">
+      <c r="G32" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="H32" s="109"/>
+      <c r="H32" s="107"/>
     </row>
     <row r="33" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
@@ -3664,7 +3692,7 @@
       </c>
     </row>
     <row r="37" spans="2:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="B37" s="110" t="s">
+      <c r="B37" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C37" s="19">
@@ -3686,7 +3714,7 @@
       </c>
     </row>
     <row r="38" spans="2:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="B38" s="110"/>
+      <c r="B38" s="102"/>
       <c r="C38" s="59">
         <v>0</v>
       </c>
@@ -3703,7 +3731,9 @@
         <f>C38*G33+D38*G34+E38*G35</f>
         <v>7</v>
       </c>
-      <c r="H38" s="23"/>
+      <c r="H38" s="23">
+        <v>4</v>
+      </c>
     </row>
     <row r="39" spans="2:8" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="8"/>
@@ -3711,13 +3741,19 @@
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
       <c r="F39" s="72"/>
-      <c r="G39" s="102" t="s">
+      <c r="G39" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="H39" s="103"/>
+      <c r="H39" s="116"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="F26:I26"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="F6:I6"/>
     <mergeCell ref="B10:B11"/>
@@ -3732,12 +3768,6 @@
     <mergeCell ref="P13:Q13"/>
     <mergeCell ref="K17:Q17"/>
     <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="O26:Q26"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="F26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="S1" r:id="rId1" xr:uid="{A34BF2FF-0E95-C94E-B3C7-66CDDE6AA8BB}"/>
@@ -3804,7 +3834,7 @@
       <c r="R3" s="27"/>
     </row>
     <row r="4" spans="1:20" ht="19" x14ac:dyDescent="0.25">
-      <c r="B4" s="111" t="s">
+      <c r="B4" s="103" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="123"/>
@@ -3813,16 +3843,16 @@
       <c r="F4" s="123"/>
       <c r="G4" s="123"/>
       <c r="H4" s="124"/>
-      <c r="K4" s="114" t="s">
+      <c r="K4" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="122"/>
+      <c r="L4" s="109"/>
+      <c r="M4" s="109"/>
+      <c r="N4" s="109"/>
+      <c r="O4" s="109"/>
+      <c r="P4" s="109"/>
+      <c r="Q4" s="109"/>
+      <c r="R4" s="121"/>
     </row>
     <row r="5" spans="1:20" ht="19" x14ac:dyDescent="0.25">
       <c r="B5" s="68">
@@ -3851,20 +3881,20 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="G6" s="108" t="s">
+      <c r="G6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="109"/>
+      <c r="H6" s="107"/>
       <c r="K6" s="4"/>
       <c r="L6" s="3"/>
       <c r="M6" s="29"/>
       <c r="N6" s="29"/>
-      <c r="O6" s="117" t="s">
+      <c r="O6" s="111" t="s">
         <v>47</v>
       </c>
-      <c r="P6" s="117"/>
-      <c r="Q6" s="117"/>
-      <c r="R6" s="121"/>
+      <c r="P6" s="111"/>
+      <c r="Q6" s="111"/>
+      <c r="R6" s="122"/>
     </row>
     <row r="7" spans="1:20" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="4"/>
@@ -3955,7 +3985,7 @@
       <c r="H10" s="71" t="s">
         <v>43</v>
       </c>
-      <c r="K10" s="119" t="s">
+      <c r="K10" s="113" t="s">
         <v>48</v>
       </c>
       <c r="L10" s="36">
@@ -3983,7 +4013,7 @@
       </c>
     </row>
     <row r="11" spans="1:20" ht="19" x14ac:dyDescent="0.25">
-      <c r="B11" s="110" t="s">
+      <c r="B11" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C11" s="19">
@@ -4002,7 +4032,7 @@
       <c r="H11" s="70">
         <v>-1</v>
       </c>
-      <c r="K11" s="119"/>
+      <c r="K11" s="113"/>
       <c r="L11" s="47">
         <v>2</v>
       </c>
@@ -4028,7 +4058,7 @@
       </c>
     </row>
     <row r="12" spans="1:20" ht="19" x14ac:dyDescent="0.25">
-      <c r="B12" s="110"/>
+      <c r="B12" s="102"/>
       <c r="C12" s="59">
         <v>1</v>
       </c>
@@ -4047,7 +4077,7 @@
         <f>C12*H7+D12*H8+E12*H9</f>
         <v>3</v>
       </c>
-      <c r="K12" s="119"/>
+      <c r="K12" s="113"/>
       <c r="L12" s="47">
         <v>1</v>
       </c>
@@ -4077,11 +4107,11 @@
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="72"/>
-      <c r="G13" s="102" t="s">
+      <c r="G13" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="103"/>
-      <c r="K13" s="119"/>
+      <c r="H13" s="116"/>
+      <c r="K13" s="113"/>
       <c r="L13" s="36">
         <v>4</v>
       </c>
@@ -4151,7 +4181,7 @@
       </c>
     </row>
     <row r="18" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B18" s="111" t="s">
+      <c r="B18" s="103" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="123"/>
@@ -4160,7 +4190,7 @@
       <c r="F18" s="123"/>
       <c r="G18" s="123"/>
       <c r="H18" s="124"/>
-      <c r="K18" s="111" t="s">
+      <c r="K18" s="103" t="s">
         <v>19</v>
       </c>
       <c r="L18" s="123"/>
@@ -4197,18 +4227,18 @@
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
-      <c r="G20" s="108" t="s">
+      <c r="G20" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="H20" s="109"/>
+      <c r="H20" s="107"/>
       <c r="K20" s="4"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
-      <c r="Q20" s="108" t="s">
+      <c r="Q20" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="R20" s="109"/>
+      <c r="R20" s="107"/>
     </row>
     <row r="21" spans="2:18" ht="19" x14ac:dyDescent="0.25">
       <c r="B21" s="4"/>
@@ -4295,7 +4325,7 @@
       </c>
     </row>
     <row r="25" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B25" s="110" t="s">
+      <c r="B25" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C25" s="19">
@@ -4326,7 +4356,7 @@
       </c>
     </row>
     <row r="26" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B26" s="110"/>
+      <c r="B26" s="102"/>
       <c r="C26" s="59">
         <v>1</v>
       </c>
@@ -4346,7 +4376,7 @@
       <c r="H26" s="77">
         <v>6</v>
       </c>
-      <c r="K26" s="110" t="s">
+      <c r="K26" s="102" t="s">
         <v>47</v>
       </c>
       <c r="L26" s="66">
@@ -4377,11 +4407,11 @@
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="72"/>
-      <c r="G27" s="102" t="s">
+      <c r="G27" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="H27" s="103"/>
-      <c r="K27" s="110"/>
+      <c r="H27" s="116"/>
+      <c r="K27" s="102"/>
       <c r="L27" s="67">
         <v>0</v>
       </c>
@@ -4410,7 +4440,7 @@
       <c r="E28" s="3"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="K28" s="110"/>
+      <c r="K28" s="102"/>
       <c r="L28" s="19">
         <v>0</v>
       </c>
@@ -4439,7 +4469,7 @@
       <c r="E29" s="3"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="K29" s="110"/>
+      <c r="K29" s="102"/>
       <c r="L29" s="19">
         <v>1</v>
       </c>
@@ -4480,7 +4510,7 @@
       </c>
     </row>
     <row r="32" spans="2:18" ht="19" x14ac:dyDescent="0.25">
-      <c r="B32" s="111" t="s">
+      <c r="B32" s="103" t="s">
         <v>17</v>
       </c>
       <c r="C32" s="123"/>
@@ -4508,10 +4538,10 @@
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
-      <c r="H34" s="108" t="s">
+      <c r="H34" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="I34" s="109"/>
+      <c r="I34" s="107"/>
     </row>
     <row r="35" spans="2:9" ht="19" x14ac:dyDescent="0.25">
       <c r="B35" s="4"/>
@@ -4571,7 +4601,7 @@
       </c>
     </row>
     <row r="40" spans="2:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="B40" s="110" t="s">
+      <c r="B40" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C40" s="66">
@@ -4596,7 +4626,7 @@
       <c r="I40" s="65"/>
     </row>
     <row r="41" spans="2:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="B41" s="110"/>
+      <c r="B41" s="102"/>
       <c r="C41" s="67">
         <v>1</v>
       </c>
@@ -4625,10 +4655,10 @@
       <c r="E42" s="9"/>
       <c r="F42" s="72"/>
       <c r="G42" s="72"/>
-      <c r="H42" s="102" t="s">
+      <c r="H42" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="I42" s="103"/>
+      <c r="I42" s="116"/>
     </row>
     <row r="43" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="44" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4638,6 +4668,14 @@
     <row r="48" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="K26:K29"/>
+    <mergeCell ref="K18:R18"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="K4:R4"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="O14:R14"/>
+    <mergeCell ref="K10:K13"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="H34:I34"/>
     <mergeCell ref="H42:I42"/>
@@ -4650,14 +4688,6 @@
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="B32:I32"/>
-    <mergeCell ref="K26:K29"/>
-    <mergeCell ref="K18:R18"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q30:R30"/>
-    <mergeCell ref="K4:R4"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="O14:R14"/>
-    <mergeCell ref="K10:K13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="T1" r:id="rId1" xr:uid="{E34E8C5F-EBFA-F74D-8879-2262033A5A5E}"/>
@@ -4724,7 +4754,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.25">
-      <c r="B4" s="111" t="s">
+      <c r="B4" s="103" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="123"/>
@@ -4737,7 +4767,7 @@
       <c r="J4" s="52"/>
       <c r="K4" s="52"/>
       <c r="L4" s="52"/>
-      <c r="N4" s="111" t="s">
+      <c r="N4" s="103" t="s">
         <v>23</v>
       </c>
       <c r="O4" s="123"/>
@@ -4775,10 +4805,10 @@
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
-      <c r="H6" s="108" t="s">
+      <c r="H6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="109"/>
+      <c r="I6" s="107"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -4786,10 +4816,10 @@
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="T6" s="108" t="s">
+      <c r="T6" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="U6" s="109"/>
+      <c r="U6" s="107"/>
     </row>
     <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="4"/>
@@ -4912,7 +4942,7 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="B12" s="110" t="s">
+      <c r="B12" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C12" s="66">
@@ -4936,7 +4966,7 @@
         <f>C12*I7+D12*I8+E12*I9+I10*F12</f>
         <v>1</v>
       </c>
-      <c r="N12" s="110" t="s">
+      <c r="N12" s="102" t="s">
         <v>47</v>
       </c>
       <c r="O12" s="66">
@@ -4962,7 +4992,7 @@
       </c>
     </row>
     <row r="13" spans="1:26" ht="19" x14ac:dyDescent="0.2">
-      <c r="B13" s="110"/>
+      <c r="B13" s="102"/>
       <c r="C13" s="67">
         <v>0</v>
       </c>
@@ -4983,7 +5013,7 @@
         <f>C13*I7+D13*I8+E13*I9+I10*F13</f>
         <v>0</v>
       </c>
-      <c r="N13" s="110"/>
+      <c r="N13" s="102"/>
       <c r="O13" s="67">
         <v>0</v>
       </c>
@@ -5006,7 +5036,7 @@
       </c>
     </row>
     <row r="14" spans="1:26" ht="19" x14ac:dyDescent="0.25">
-      <c r="B14" s="110"/>
+      <c r="B14" s="102"/>
       <c r="C14" s="19">
         <v>0</v>
       </c>
@@ -5027,7 +5057,7 @@
         <f>C14*I7+D14*I8+E14*I9+F14*I10</f>
         <v>-2</v>
       </c>
-      <c r="N14" s="110"/>
+      <c r="N14" s="102"/>
       <c r="O14" s="22"/>
       <c r="P14" s="19">
         <v>0</v>
@@ -5049,7 +5079,7 @@
       </c>
     </row>
     <row r="15" spans="1:26" ht="19" x14ac:dyDescent="0.25">
-      <c r="B15" s="110"/>
+      <c r="B15" s="102"/>
       <c r="C15" s="19">
         <v>-1</v>
       </c>
@@ -5070,7 +5100,7 @@
         <f>C15*I7+D15*I8+E15*I9+F15*I10</f>
         <v>1</v>
       </c>
-      <c r="N15" s="110"/>
+      <c r="N15" s="102"/>
       <c r="O15" s="19">
         <v>1</v>
       </c>
@@ -5141,7 +5171,7 @@
       </c>
     </row>
     <row r="20" spans="2:24" ht="19" x14ac:dyDescent="0.25">
-      <c r="B20" s="111" t="s">
+      <c r="B20" s="103" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="123"/>
@@ -5154,19 +5184,19 @@
       <c r="J20" s="123"/>
       <c r="K20" s="123"/>
       <c r="L20" s="124"/>
-      <c r="N20" s="133" t="s">
+      <c r="N20" s="136" t="s">
         <v>24</v>
       </c>
-      <c r="O20" s="134"/>
-      <c r="P20" s="134"/>
-      <c r="Q20" s="134"/>
-      <c r="R20" s="134"/>
-      <c r="S20" s="134"/>
-      <c r="T20" s="134"/>
-      <c r="U20" s="134"/>
-      <c r="V20" s="134"/>
-      <c r="W20" s="134"/>
-      <c r="X20" s="135"/>
+      <c r="O20" s="137"/>
+      <c r="P20" s="137"/>
+      <c r="Q20" s="137"/>
+      <c r="R20" s="137"/>
+      <c r="S20" s="137"/>
+      <c r="T20" s="137"/>
+      <c r="U20" s="137"/>
+      <c r="V20" s="137"/>
+      <c r="W20" s="137"/>
+      <c r="X20" s="138"/>
     </row>
     <row r="21" spans="2:24" ht="19" x14ac:dyDescent="0.25">
       <c r="B21" s="68">
@@ -5195,24 +5225,24 @@
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
-      <c r="H22" s="108" t="s">
+      <c r="H22" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="I22" s="108"/>
-      <c r="J22" s="108"/>
-      <c r="K22" s="108"/>
-      <c r="L22" s="109"/>
+      <c r="I22" s="106"/>
+      <c r="J22" s="106"/>
+      <c r="K22" s="106"/>
+      <c r="L22" s="107"/>
       <c r="N22" s="4"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
-      <c r="T22" s="108" t="s">
+      <c r="T22" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="U22" s="108"/>
-      <c r="V22" s="108"/>
-      <c r="W22" s="108"/>
-      <c r="X22" s="109"/>
+      <c r="U22" s="106"/>
+      <c r="V22" s="106"/>
+      <c r="W22" s="106"/>
+      <c r="X22" s="107"/>
     </row>
     <row r="23" spans="2:24" ht="19" x14ac:dyDescent="0.25">
       <c r="B23" s="4"/>
@@ -5394,7 +5424,7 @@
       <c r="X27" s="80"/>
     </row>
     <row r="28" spans="2:24" ht="19" x14ac:dyDescent="0.25">
-      <c r="B28" s="110" t="s">
+      <c r="B28" s="102" t="s">
         <v>47</v>
       </c>
       <c r="C28" s="66">
@@ -5429,7 +5459,7 @@
         <f>C28*L23+D28*L24+E28*L25+F28*L26</f>
         <v>7</v>
       </c>
-      <c r="N28" s="110" t="s">
+      <c r="N28" s="102" t="s">
         <v>47</v>
       </c>
       <c r="O28" s="66">
@@ -5466,7 +5496,7 @@
       </c>
     </row>
     <row r="29" spans="2:24" ht="19" x14ac:dyDescent="0.2">
-      <c r="B29" s="110"/>
+      <c r="B29" s="102"/>
       <c r="C29" s="67">
         <v>13</v>
       </c>
@@ -5499,7 +5529,7 @@
         <f>C29*L23+D29*L24+E29*L25+F29*L26</f>
         <v>16</v>
       </c>
-      <c r="N29" s="110"/>
+      <c r="N29" s="102"/>
       <c r="O29" s="67">
         <v>0</v>
       </c>
@@ -5540,14 +5570,14 @@
       <c r="E30" s="9"/>
       <c r="F30" s="72"/>
       <c r="G30" s="72"/>
-      <c r="H30" s="102" t="s">
+      <c r="H30" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="I30" s="102"/>
-      <c r="J30" s="102"/>
-      <c r="K30" s="102"/>
-      <c r="L30" s="103"/>
-      <c r="N30" s="110"/>
+      <c r="I30" s="115"/>
+      <c r="J30" s="115"/>
+      <c r="K30" s="115"/>
+      <c r="L30" s="116"/>
+      <c r="N30" s="102"/>
       <c r="O30" s="19">
         <v>1</v>
       </c>
@@ -5588,7 +5618,7 @@
       <c r="E31" s="3"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
-      <c r="N31" s="110"/>
+      <c r="N31" s="102"/>
       <c r="O31" s="19">
         <v>1</v>
       </c>
@@ -5629,7 +5659,7 @@
       <c r="E32" s="3"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-      <c r="N32" s="110"/>
+      <c r="N32" s="102"/>
       <c r="O32" s="19">
         <v>1</v>
       </c>
@@ -5674,28 +5704,28 @@
       <c r="Q33" s="9"/>
       <c r="R33" s="72"/>
       <c r="S33" s="72"/>
-      <c r="T33" s="102" t="s">
+      <c r="T33" s="115" t="s">
         <v>49</v>
       </c>
-      <c r="U33" s="102"/>
-      <c r="V33" s="102"/>
-      <c r="W33" s="102"/>
-      <c r="X33" s="103"/>
+      <c r="U33" s="115"/>
+      <c r="V33" s="115"/>
+      <c r="W33" s="115"/>
+      <c r="X33" s="116"/>
     </row>
     <row r="34" spans="2:24" ht="19" x14ac:dyDescent="0.25">
-      <c r="B34" s="136" t="s">
+      <c r="B34" s="129" t="s">
         <v>22</v>
       </c>
-      <c r="C34" s="137"/>
-      <c r="D34" s="137"/>
-      <c r="E34" s="137"/>
-      <c r="F34" s="137"/>
-      <c r="G34" s="137"/>
-      <c r="H34" s="137"/>
-      <c r="I34" s="137"/>
-      <c r="J34" s="137"/>
-      <c r="K34" s="137"/>
-      <c r="L34" s="138"/>
+      <c r="C34" s="130"/>
+      <c r="D34" s="130"/>
+      <c r="E34" s="130"/>
+      <c r="F34" s="130"/>
+      <c r="G34" s="130"/>
+      <c r="H34" s="130"/>
+      <c r="I34" s="130"/>
+      <c r="J34" s="130"/>
+      <c r="K34" s="130"/>
+      <c r="L34" s="131"/>
     </row>
     <row r="35" spans="2:24" ht="19" x14ac:dyDescent="0.25">
       <c r="B35" s="92">
@@ -5714,13 +5744,13 @@
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
-      <c r="H36" s="108" t="s">
+      <c r="H36" s="106" t="s">
         <v>48</v>
       </c>
-      <c r="I36" s="108"/>
-      <c r="J36" s="108"/>
-      <c r="K36" s="108"/>
-      <c r="L36" s="129"/>
+      <c r="I36" s="106"/>
+      <c r="J36" s="106"/>
+      <c r="K36" s="106"/>
+      <c r="L36" s="132"/>
     </row>
     <row r="37" spans="2:24" ht="19" x14ac:dyDescent="0.25">
       <c r="B37" s="94"/>
@@ -5829,7 +5859,7 @@
       <c r="M41" s="15"/>
     </row>
     <row r="42" spans="2:24" ht="19" x14ac:dyDescent="0.25">
-      <c r="B42" s="130" t="s">
+      <c r="B42" s="133" t="s">
         <v>47</v>
       </c>
       <c r="C42" s="66">
@@ -5867,7 +5897,7 @@
       <c r="P42" s="90"/>
     </row>
     <row r="43" spans="2:24" ht="19" x14ac:dyDescent="0.2">
-      <c r="B43" s="130"/>
+      <c r="B43" s="133"/>
       <c r="C43" s="67">
         <v>3</v>
       </c>
@@ -5911,21 +5941,16 @@
       <c r="E44" s="100"/>
       <c r="F44" s="101"/>
       <c r="G44" s="101"/>
-      <c r="H44" s="131" t="s">
+      <c r="H44" s="134" t="s">
         <v>49</v>
       </c>
-      <c r="I44" s="131"/>
-      <c r="J44" s="131"/>
-      <c r="K44" s="131"/>
-      <c r="L44" s="132"/>
+      <c r="I44" s="134"/>
+      <c r="J44" s="134"/>
+      <c r="K44" s="134"/>
+      <c r="L44" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="H30:L30"/>
-    <mergeCell ref="B20:L20"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="H36:L36"/>
     <mergeCell ref="B42:B43"/>
     <mergeCell ref="H44:L44"/>
     <mergeCell ref="N4:U4"/>
@@ -5941,6 +5966,11 @@
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="B28:B29"/>
+    <mergeCell ref="H22:L22"/>
+    <mergeCell ref="H30:L30"/>
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="B34:L34"/>
+    <mergeCell ref="H36:L36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Z1" r:id="rId1" xr:uid="{45024357-32C1-ED48-9305-5D55817EC8E5}"/>

</xml_diff>